<commit_message>
Improved model period matrix
</commit_message>
<xml_diff>
--- a/annual/Annual_Jevons_Index_Results.xlsx
+++ b/annual/Annual_Jevons_Index_Results.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Adjacent Years" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="All Year Pairs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Annual_Price_Data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Model_Period_Matrix" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14369,6 +14370,2763 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:EW8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 128GB</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 256GB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 64GB</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 Pro 64GB</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 Pro Max 256GB</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 Pro Max 512GB</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 11 Pro Max 64GB</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 128GB</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 256GB</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 64GB</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 Pro 128GB</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 Pro Max 128GB</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 Pro Max 256GB</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 Pro Max 512GB</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 mini 128GB</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 mini 256GB</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 12 mini 64GB</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 128GB</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 256GB</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 512GB</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 Pro 128GB</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 Pro Max 128GB</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 Pro Max 256GB</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 Pro Max 512GB</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 mini 128GB</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 mini 256GB</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 13 mini 512GB</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 128GB</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 256GB</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 512GB</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Plus 128GB</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Plus 256GB</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Plus 512GB</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Pro 128GB</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Pro Max 128GB</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Pro Max 256GB</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 14 Pro Max 512GB</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 128GB</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 256GB</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 512GB</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 Plus 128GB</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 Plus 256GB</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 Plus 512GB</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 Pro 128GB</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 Pro Max 256GB</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 15 Pro Max 512GB</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 128GB</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 256GB</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 512GB</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 Plus 128GB</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 Plus 256GB</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 Plus 512GB</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 Pro 128GB</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 Pro Max 256GB</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone 16 Pro Max 512GB</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone X 64GB</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XR 128GB</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XR 256GB</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XR 64GB</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XS 256GB</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XS 512GB</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XS 64GB</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XS Max 256GB</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XS Max 512GB</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>Apple - iPhone XS Max 64GB</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 10 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 10T 5G 256GB</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 11 256GB</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 12 256GB</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 12R 256GB</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 7 Pro 5G 256GB</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 8 128GB</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 8 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 8T 256GB</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 9 128GB</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus 9 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus Nord 2 5G 128GB</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus Nord 2T 128GB</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus Nord CE 3 Lite 256GB</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus Nord N10 5G 128GB</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus Nord N100 5G 64GB</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus Nord N200 64GB</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>OnePlus - OnePlus Nord N30 5G 128GB</t>
+        </is>
+      </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - A60 128GB</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - A60 256GB</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - A80 256GB</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Find N2 Flip 256GB</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Find X5 256GB</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Find X5 Pro 256GB</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Find X8 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno10 5G 256GB</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno10 Pro 5G 256GB</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno11 F 256GB</t>
+        </is>
+      </c>
+      <c r="DC1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno11 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno12 256GB</t>
+        </is>
+      </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno12 F 4G 256GB</t>
+        </is>
+      </c>
+      <c r="DF1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno12 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="DG1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno13 256GB</t>
+        </is>
+      </c>
+      <c r="DH1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno13 F 4G 256GB</t>
+        </is>
+      </c>
+      <c r="DI1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno13 Pro 512GB</t>
+        </is>
+      </c>
+      <c r="DJ1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno7 5G 128GB</t>
+        </is>
+      </c>
+      <c r="DK1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno7 5G 256GB</t>
+        </is>
+      </c>
+      <c r="DL1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno7 Pro 5G 256GB</t>
+        </is>
+      </c>
+      <c r="DM1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno8 5G 128GB</t>
+        </is>
+      </c>
+      <c r="DN1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno8 5G 256GB</t>
+        </is>
+      </c>
+      <c r="DO1" s="1" t="inlineStr">
+        <is>
+          <t>Oppo - Reno8 Pro 5G 256GB</t>
+        </is>
+      </c>
+      <c r="DP1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy A04 64GB</t>
+        </is>
+      </c>
+      <c r="DQ1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy A24 128GB</t>
+        </is>
+      </c>
+      <c r="DR1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy A34 256GB</t>
+        </is>
+      </c>
+      <c r="DS1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy A54 128GB</t>
+        </is>
+      </c>
+      <c r="DT1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy A54 256GB</t>
+        </is>
+      </c>
+      <c r="DU1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Note 10 256GB</t>
+        </is>
+      </c>
+      <c r="DV1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Note 10+ 256GB</t>
+        </is>
+      </c>
+      <c r="DW1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Note 10+ 512GB</t>
+        </is>
+      </c>
+      <c r="DX1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Note 20 128GB</t>
+        </is>
+      </c>
+      <c r="DY1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Note 20 Ultra 128GB</t>
+        </is>
+      </c>
+      <c r="DZ1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S22 128GB</t>
+        </is>
+      </c>
+      <c r="EA1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S22 256GB</t>
+        </is>
+      </c>
+      <c r="EB1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S22 Ultra 128GB</t>
+        </is>
+      </c>
+      <c r="EC1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S22 Ultra 256GB</t>
+        </is>
+      </c>
+      <c r="ED1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S22+ 128GB</t>
+        </is>
+      </c>
+      <c r="EE1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S22+ 256GB</t>
+        </is>
+      </c>
+      <c r="EF1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S23 128GB</t>
+        </is>
+      </c>
+      <c r="EG1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S23 256GB</t>
+        </is>
+      </c>
+      <c r="EH1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S23 Ultra 256GB</t>
+        </is>
+      </c>
+      <c r="EI1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S23+ 256GB</t>
+        </is>
+      </c>
+      <c r="EJ1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S24 128GB</t>
+        </is>
+      </c>
+      <c r="EK1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S24 256GB</t>
+        </is>
+      </c>
+      <c r="EL1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S24 Ultra 256GB</t>
+        </is>
+      </c>
+      <c r="EM1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy S24+ 256GB</t>
+        </is>
+      </c>
+      <c r="EN1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Xcover 5 64GB</t>
+        </is>
+      </c>
+      <c r="EO1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Xcover 6 Pro 128GB</t>
+        </is>
+      </c>
+      <c r="EP1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Z Flip 4 256GB</t>
+        </is>
+      </c>
+      <c r="EQ1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Z Flip 4 512GB</t>
+        </is>
+      </c>
+      <c r="ER1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Z Flip 5 256GB</t>
+        </is>
+      </c>
+      <c r="ES1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Z Flip 5 512GB</t>
+        </is>
+      </c>
+      <c r="ET1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Z Fold 4 256GB</t>
+        </is>
+      </c>
+      <c r="EU1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Z Fold 4 512GB</t>
+        </is>
+      </c>
+      <c r="EV1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Z Fold 5 256GB</t>
+        </is>
+      </c>
+      <c r="EW1" s="1" t="inlineStr">
+        <is>
+          <t>Samsung - Galaxy Z Fold 5 512GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>2018→2019</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="n">
+        <v>-0.01306433149200625</v>
+      </c>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="n">
+        <v>-0.04956712224988813</v>
+      </c>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr"/>
+      <c r="CC2" t="inlineStr"/>
+      <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="inlineStr"/>
+      <c r="CH2" t="inlineStr"/>
+      <c r="CI2" t="inlineStr"/>
+      <c r="CJ2" t="inlineStr"/>
+      <c r="CK2" t="inlineStr"/>
+      <c r="CL2" t="inlineStr"/>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="inlineStr"/>
+      <c r="CV2" t="inlineStr"/>
+      <c r="CW2" t="inlineStr"/>
+      <c r="CX2" t="inlineStr"/>
+      <c r="CY2" t="inlineStr"/>
+      <c r="CZ2" t="inlineStr"/>
+      <c r="DA2" t="inlineStr"/>
+      <c r="DB2" t="inlineStr"/>
+      <c r="DC2" t="inlineStr"/>
+      <c r="DD2" t="inlineStr"/>
+      <c r="DE2" t="inlineStr"/>
+      <c r="DF2" t="inlineStr"/>
+      <c r="DG2" t="inlineStr"/>
+      <c r="DH2" t="inlineStr"/>
+      <c r="DI2" t="inlineStr"/>
+      <c r="DJ2" t="inlineStr"/>
+      <c r="DK2" t="inlineStr"/>
+      <c r="DL2" t="inlineStr"/>
+      <c r="DM2" t="inlineStr"/>
+      <c r="DN2" t="inlineStr"/>
+      <c r="DO2" t="inlineStr"/>
+      <c r="DP2" t="inlineStr"/>
+      <c r="DQ2" t="inlineStr"/>
+      <c r="DR2" t="inlineStr"/>
+      <c r="DS2" t="inlineStr"/>
+      <c r="DT2" t="inlineStr"/>
+      <c r="DU2" t="inlineStr"/>
+      <c r="DV2" t="inlineStr"/>
+      <c r="DW2" t="inlineStr"/>
+      <c r="DX2" t="inlineStr"/>
+      <c r="DY2" t="inlineStr"/>
+      <c r="DZ2" t="inlineStr"/>
+      <c r="EA2" t="inlineStr"/>
+      <c r="EB2" t="inlineStr"/>
+      <c r="EC2" t="inlineStr"/>
+      <c r="ED2" t="inlineStr"/>
+      <c r="EE2" t="inlineStr"/>
+      <c r="EF2" t="inlineStr"/>
+      <c r="EG2" t="inlineStr"/>
+      <c r="EH2" t="inlineStr"/>
+      <c r="EI2" t="inlineStr"/>
+      <c r="EJ2" t="inlineStr"/>
+      <c r="EK2" t="inlineStr"/>
+      <c r="EL2" t="inlineStr"/>
+      <c r="EM2" t="inlineStr"/>
+      <c r="EN2" t="inlineStr"/>
+      <c r="EO2" t="inlineStr"/>
+      <c r="EP2" t="inlineStr"/>
+      <c r="EQ2" t="inlineStr"/>
+      <c r="ER2" t="inlineStr"/>
+      <c r="ES2" t="inlineStr"/>
+      <c r="ET2" t="inlineStr"/>
+      <c r="EU2" t="inlineStr"/>
+      <c r="EV2" t="inlineStr"/>
+      <c r="EW2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>2019→2020</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.06293881665941203</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-0.1225211963430617</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-0.129162158949538</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.183686177529748</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.1785099548872013</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.1414916366085128</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-0.1577928979229251</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.114032413478764</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-0.1240625885866109</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
+      <c r="BI3" t="inlineStr"/>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="n">
+        <v>-0.3407933673449515</v>
+      </c>
+      <c r="BS3" t="n">
+        <v>-0.3086710017863972</v>
+      </c>
+      <c r="BT3" t="n">
+        <v>-0.3131173448846134</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>-0.4627896369436462</v>
+      </c>
+      <c r="BV3" t="inlineStr"/>
+      <c r="BW3" t="n">
+        <v>-0.4452620434150143</v>
+      </c>
+      <c r="BX3" t="n">
+        <v>-0.6095780626376852</v>
+      </c>
+      <c r="BY3" t="n">
+        <v>-0.5502663540063502</v>
+      </c>
+      <c r="BZ3" t="n">
+        <v>-0.5992555238928921</v>
+      </c>
+      <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr"/>
+      <c r="CC3" t="inlineStr"/>
+      <c r="CD3" t="inlineStr"/>
+      <c r="CE3" t="inlineStr"/>
+      <c r="CF3" t="inlineStr"/>
+      <c r="CG3" t="inlineStr"/>
+      <c r="CH3" t="inlineStr"/>
+      <c r="CI3" t="inlineStr"/>
+      <c r="CJ3" t="inlineStr"/>
+      <c r="CK3" t="inlineStr"/>
+      <c r="CL3" t="inlineStr"/>
+      <c r="CM3" t="inlineStr"/>
+      <c r="CN3" t="inlineStr"/>
+      <c r="CO3" t="inlineStr"/>
+      <c r="CP3" t="inlineStr"/>
+      <c r="CQ3" t="inlineStr"/>
+      <c r="CR3" t="inlineStr"/>
+      <c r="CS3" t="inlineStr"/>
+      <c r="CT3" t="inlineStr"/>
+      <c r="CU3" t="inlineStr"/>
+      <c r="CV3" t="inlineStr"/>
+      <c r="CW3" t="inlineStr"/>
+      <c r="CX3" t="inlineStr"/>
+      <c r="CY3" t="inlineStr"/>
+      <c r="CZ3" t="inlineStr"/>
+      <c r="DA3" t="inlineStr"/>
+      <c r="DB3" t="inlineStr"/>
+      <c r="DC3" t="inlineStr"/>
+      <c r="DD3" t="inlineStr"/>
+      <c r="DE3" t="inlineStr"/>
+      <c r="DF3" t="inlineStr"/>
+      <c r="DG3" t="inlineStr"/>
+      <c r="DH3" t="inlineStr"/>
+      <c r="DI3" t="inlineStr"/>
+      <c r="DJ3" t="inlineStr"/>
+      <c r="DK3" t="inlineStr"/>
+      <c r="DL3" t="inlineStr"/>
+      <c r="DM3" t="inlineStr"/>
+      <c r="DN3" t="inlineStr"/>
+      <c r="DO3" t="inlineStr"/>
+      <c r="DP3" t="inlineStr"/>
+      <c r="DQ3" t="inlineStr"/>
+      <c r="DR3" t="inlineStr"/>
+      <c r="DS3" t="inlineStr"/>
+      <c r="DT3" t="inlineStr"/>
+      <c r="DU3" t="n">
+        <v>-0.1489026953209898</v>
+      </c>
+      <c r="DV3" t="inlineStr"/>
+      <c r="DW3" t="n">
+        <v>-0.1066942436118605</v>
+      </c>
+      <c r="DX3" t="inlineStr"/>
+      <c r="DY3" t="inlineStr"/>
+      <c r="DZ3" t="inlineStr"/>
+      <c r="EA3" t="inlineStr"/>
+      <c r="EB3" t="inlineStr"/>
+      <c r="EC3" t="inlineStr"/>
+      <c r="ED3" t="inlineStr"/>
+      <c r="EE3" t="inlineStr"/>
+      <c r="EF3" t="inlineStr"/>
+      <c r="EG3" t="inlineStr"/>
+      <c r="EH3" t="inlineStr"/>
+      <c r="EI3" t="inlineStr"/>
+      <c r="EJ3" t="inlineStr"/>
+      <c r="EK3" t="inlineStr"/>
+      <c r="EL3" t="inlineStr"/>
+      <c r="EM3" t="inlineStr"/>
+      <c r="EN3" t="inlineStr"/>
+      <c r="EO3" t="inlineStr"/>
+      <c r="EP3" t="inlineStr"/>
+      <c r="EQ3" t="inlineStr"/>
+      <c r="ER3" t="inlineStr"/>
+      <c r="ES3" t="inlineStr"/>
+      <c r="ET3" t="inlineStr"/>
+      <c r="EU3" t="inlineStr"/>
+      <c r="EV3" t="inlineStr"/>
+      <c r="EW3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>2020→2021</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.2282556341203037</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-0.2034576153710894</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.2422176407004635</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.322651716791662</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.3253506616160706</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.3043198954269997</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-0.2986708121509514</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.3729528231789301</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-0.3277382973490299</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="n">
+        <v>-0.2132014833282403</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>-0.2270777887459152</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>-0.2588652408947612</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>-0.286224040896113</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>-0.2079857863755317</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>-0.3061094989811517</v>
+      </c>
+      <c r="BX4" t="n">
+        <v>-0.246017086023131</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>-0.1996556113079464</v>
+      </c>
+      <c r="BZ4" t="n">
+        <v>-0.2512739343818753</v>
+      </c>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr"/>
+      <c r="CC4" t="inlineStr"/>
+      <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="n">
+        <v>-0.3895755518330182</v>
+      </c>
+      <c r="CG4" t="inlineStr"/>
+      <c r="CH4" t="n">
+        <v>-0.1914277158109199</v>
+      </c>
+      <c r="CI4" t="inlineStr"/>
+      <c r="CJ4" t="inlineStr"/>
+      <c r="CK4" t="inlineStr"/>
+      <c r="CL4" t="inlineStr"/>
+      <c r="CM4" t="inlineStr"/>
+      <c r="CN4" t="inlineStr"/>
+      <c r="CO4" t="inlineStr"/>
+      <c r="CP4" t="inlineStr"/>
+      <c r="CQ4" t="inlineStr"/>
+      <c r="CR4" t="inlineStr"/>
+      <c r="CS4" t="inlineStr"/>
+      <c r="CT4" t="inlineStr"/>
+      <c r="CU4" t="inlineStr"/>
+      <c r="CV4" t="inlineStr"/>
+      <c r="CW4" t="inlineStr"/>
+      <c r="CX4" t="inlineStr"/>
+      <c r="CY4" t="inlineStr"/>
+      <c r="CZ4" t="inlineStr"/>
+      <c r="DA4" t="inlineStr"/>
+      <c r="DB4" t="inlineStr"/>
+      <c r="DC4" t="inlineStr"/>
+      <c r="DD4" t="inlineStr"/>
+      <c r="DE4" t="inlineStr"/>
+      <c r="DF4" t="inlineStr"/>
+      <c r="DG4" t="inlineStr"/>
+      <c r="DH4" t="inlineStr"/>
+      <c r="DI4" t="inlineStr"/>
+      <c r="DJ4" t="inlineStr"/>
+      <c r="DK4" t="inlineStr"/>
+      <c r="DL4" t="inlineStr"/>
+      <c r="DM4" t="inlineStr"/>
+      <c r="DN4" t="inlineStr"/>
+      <c r="DO4" t="inlineStr"/>
+      <c r="DP4" t="inlineStr"/>
+      <c r="DQ4" t="inlineStr"/>
+      <c r="DR4" t="inlineStr"/>
+      <c r="DS4" t="inlineStr"/>
+      <c r="DT4" t="inlineStr"/>
+      <c r="DU4" t="n">
+        <v>-0.3295678504660762</v>
+      </c>
+      <c r="DV4" t="n">
+        <v>-0.3708112829294032</v>
+      </c>
+      <c r="DW4" t="n">
+        <v>-0.3681537247473452</v>
+      </c>
+      <c r="DX4" t="inlineStr"/>
+      <c r="DY4" t="n">
+        <v>-0.146750390060121</v>
+      </c>
+      <c r="DZ4" t="inlineStr"/>
+      <c r="EA4" t="inlineStr"/>
+      <c r="EB4" t="inlineStr"/>
+      <c r="EC4" t="inlineStr"/>
+      <c r="ED4" t="inlineStr"/>
+      <c r="EE4" t="inlineStr"/>
+      <c r="EF4" t="inlineStr"/>
+      <c r="EG4" t="inlineStr"/>
+      <c r="EH4" t="inlineStr"/>
+      <c r="EI4" t="inlineStr"/>
+      <c r="EJ4" t="inlineStr"/>
+      <c r="EK4" t="inlineStr"/>
+      <c r="EL4" t="inlineStr"/>
+      <c r="EM4" t="inlineStr"/>
+      <c r="EN4" t="inlineStr"/>
+      <c r="EO4" t="inlineStr"/>
+      <c r="EP4" t="inlineStr"/>
+      <c r="EQ4" t="inlineStr"/>
+      <c r="ER4" t="inlineStr"/>
+      <c r="ES4" t="inlineStr"/>
+      <c r="ET4" t="inlineStr"/>
+      <c r="EU4" t="inlineStr"/>
+      <c r="EV4" t="inlineStr"/>
+      <c r="EW4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>2021→2022</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-0.3736485907697782</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.3702641970659792</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.3693684703960916</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.3573642545004212</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.2870746726961686</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-0.3742371436426941</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-0.2937705878646524</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.2655157324513366</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-0.3188493733498277</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-0.3168996293740189</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-0.3532083149953218</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-0.3639036499142243</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-0.4584363151381394</v>
+      </c>
+      <c r="O5" t="n">
+        <v>-0.513047326792158</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-0.5472978542167839</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>-0.4725284620855765</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-0.4213899302603075</v>
+      </c>
+      <c r="S5" t="n">
+        <v>-0.5002778889068837</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-0.3282062330423665</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-0.3388327247585519</v>
+      </c>
+      <c r="V5" t="n">
+        <v>-0.3450289998921621</v>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="n">
+        <v>-0.18485691094694</v>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="n">
+        <v>-0.2106562615141359</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>-0.23863553089343</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>-0.119249067350907</v>
+      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="n">
+        <v>-0.3707495637726481</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>-0.3136779342916558</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>-0.3374096159361573</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>-0.3190736227549138</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>-0.2763837230319135</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>-0.3235966064100024</v>
+      </c>
+      <c r="BX5" t="n">
+        <v>-0.3109642466236799</v>
+      </c>
+      <c r="BY5" t="n">
+        <v>-0.254214876240856</v>
+      </c>
+      <c r="BZ5" t="n">
+        <v>-0.3207469064025599</v>
+      </c>
+      <c r="CA5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr"/>
+      <c r="CC5" t="inlineStr"/>
+      <c r="CD5" t="inlineStr"/>
+      <c r="CE5" t="inlineStr"/>
+      <c r="CF5" t="n">
+        <v>-0.1352672280172778</v>
+      </c>
+      <c r="CG5" t="n">
+        <v>-0.263744907255048</v>
+      </c>
+      <c r="CH5" t="n">
+        <v>-0.2625914883747145</v>
+      </c>
+      <c r="CI5" t="inlineStr"/>
+      <c r="CJ5" t="n">
+        <v>-0.3993261640133836</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>-0.3974593763367151</v>
+      </c>
+      <c r="CL5" t="inlineStr"/>
+      <c r="CM5" t="inlineStr"/>
+      <c r="CN5" t="inlineStr"/>
+      <c r="CO5" t="n">
+        <v>-0.1975652691832481</v>
+      </c>
+      <c r="CP5" t="n">
+        <v>-0.0669319330308058</v>
+      </c>
+      <c r="CQ5" t="n">
+        <v>-0.1544142909116859</v>
+      </c>
+      <c r="CR5" t="inlineStr"/>
+      <c r="CS5" t="inlineStr"/>
+      <c r="CT5" t="inlineStr"/>
+      <c r="CU5" t="inlineStr"/>
+      <c r="CV5" t="inlineStr"/>
+      <c r="CW5" t="inlineStr"/>
+      <c r="CX5" t="inlineStr"/>
+      <c r="CY5" t="inlineStr"/>
+      <c r="CZ5" t="inlineStr"/>
+      <c r="DA5" t="inlineStr"/>
+      <c r="DB5" t="inlineStr"/>
+      <c r="DC5" t="inlineStr"/>
+      <c r="DD5" t="inlineStr"/>
+      <c r="DE5" t="inlineStr"/>
+      <c r="DF5" t="inlineStr"/>
+      <c r="DG5" t="inlineStr"/>
+      <c r="DH5" t="inlineStr"/>
+      <c r="DI5" t="inlineStr"/>
+      <c r="DJ5" t="inlineStr"/>
+      <c r="DK5" t="inlineStr"/>
+      <c r="DL5" t="inlineStr"/>
+      <c r="DM5" t="inlineStr"/>
+      <c r="DN5" t="inlineStr"/>
+      <c r="DO5" t="inlineStr"/>
+      <c r="DP5" t="inlineStr"/>
+      <c r="DQ5" t="inlineStr"/>
+      <c r="DR5" t="inlineStr"/>
+      <c r="DS5" t="inlineStr"/>
+      <c r="DT5" t="inlineStr"/>
+      <c r="DU5" t="n">
+        <v>-0.3673146384342587</v>
+      </c>
+      <c r="DV5" t="n">
+        <v>-0.2903445662109796</v>
+      </c>
+      <c r="DW5" t="n">
+        <v>-0.1730260783822581</v>
+      </c>
+      <c r="DX5" t="n">
+        <v>-0.3097855275552117</v>
+      </c>
+      <c r="DY5" t="n">
+        <v>-0.3559742449307182</v>
+      </c>
+      <c r="DZ5" t="inlineStr"/>
+      <c r="EA5" t="inlineStr"/>
+      <c r="EB5" t="inlineStr"/>
+      <c r="EC5" t="inlineStr"/>
+      <c r="ED5" t="inlineStr"/>
+      <c r="EE5" t="inlineStr"/>
+      <c r="EF5" t="inlineStr"/>
+      <c r="EG5" t="inlineStr"/>
+      <c r="EH5" t="inlineStr"/>
+      <c r="EI5" t="inlineStr"/>
+      <c r="EJ5" t="inlineStr"/>
+      <c r="EK5" t="inlineStr"/>
+      <c r="EL5" t="inlineStr"/>
+      <c r="EM5" t="inlineStr"/>
+      <c r="EN5" t="inlineStr"/>
+      <c r="EO5" t="inlineStr"/>
+      <c r="EP5" t="inlineStr"/>
+      <c r="EQ5" t="inlineStr"/>
+      <c r="ER5" t="inlineStr"/>
+      <c r="ES5" t="inlineStr"/>
+      <c r="ET5" t="inlineStr"/>
+      <c r="EU5" t="inlineStr"/>
+      <c r="EV5" t="inlineStr"/>
+      <c r="EW5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2022→2023</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.1954663828663232</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-0.1873646607772681</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.2081105036982454</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.23524985425734</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.2569489929626378</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-0.2156324200642139</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-0.2383222482936498</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.2146465333931573</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-0.2414855560010327</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-0.3646028128330983</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-0.3664714960108917</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-0.3512088354145577</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-0.3287036220579154</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-0.3071772420273451</v>
+      </c>
+      <c r="P6" t="n">
+        <v>-0.2949126669271314</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-0.2718793465468972</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-0.2883357106199771</v>
+      </c>
+      <c r="S6" t="n">
+        <v>-0.32254482366994</v>
+      </c>
+      <c r="T6" t="n">
+        <v>-0.3401805615463056</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-0.3277465438653415</v>
+      </c>
+      <c r="V6" t="n">
+        <v>-0.3461236941733308</v>
+      </c>
+      <c r="W6" t="n">
+        <v>-0.2772793449718698</v>
+      </c>
+      <c r="X6" t="n">
+        <v>-0.2748282759106493</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>-0.2411402384265724</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>-0.4084783209580376</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>-0.3743433383366277</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>-0.4551683281391279</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>-0.4678332091340573</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>-0.4173281727205351</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>-0.3557424242991392</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>-0.2614822004627158</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>-0.2603466722793479</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>-0.2056278224714729</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>-0.1944609350801416</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>-0.2159640042368292</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>-0.2722598232267783</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>-0.2308090441642285</v>
+      </c>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="n">
+        <v>-0.2210304360827742</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>-0.2786708512585268</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>-0.2350184264639044</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>-0.2501029807664965</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>-0.2925471573678831</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>-0.308241932444929</v>
+      </c>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
+      <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="n">
+        <v>-0.1146661488329634</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>-0.144873026980993</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>-0.1313318501468785</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>-0.1655478004438455</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>-0.1831230345281778</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>-0.1746697626898248</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>-0.1980129368992793</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>-0.1554021422970902</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>-0.1240671596019673</v>
+      </c>
+      <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="n">
+        <v>0.003217343988422883</v>
+      </c>
+      <c r="CG6" t="n">
+        <v>-0.1656438713257655</v>
+      </c>
+      <c r="CH6" t="n">
+        <v>-0.164467445741499</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>-0.1321075945540118</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>-0.4548076529128835</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>-0.3135066222284033</v>
+      </c>
+      <c r="CL6" t="n">
+        <v>-0.04968218543067149</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>-0.2900528093529147</v>
+      </c>
+      <c r="CN6" t="inlineStr"/>
+      <c r="CO6" t="n">
+        <v>-0.2738667811977766</v>
+      </c>
+      <c r="CP6" t="n">
+        <v>-0.2596208606662911</v>
+      </c>
+      <c r="CQ6" t="n">
+        <v>-0.3519147343662361</v>
+      </c>
+      <c r="CR6" t="inlineStr"/>
+      <c r="CS6" t="inlineStr"/>
+      <c r="CT6" t="inlineStr"/>
+      <c r="CU6" t="inlineStr"/>
+      <c r="CV6" t="inlineStr"/>
+      <c r="CW6" t="n">
+        <v>-0.1895150403035997</v>
+      </c>
+      <c r="CX6" t="n">
+        <v>-0.369793697109384</v>
+      </c>
+      <c r="CY6" t="inlineStr"/>
+      <c r="CZ6" t="inlineStr"/>
+      <c r="DA6" t="inlineStr"/>
+      <c r="DB6" t="inlineStr"/>
+      <c r="DC6" t="inlineStr"/>
+      <c r="DD6" t="inlineStr"/>
+      <c r="DE6" t="inlineStr"/>
+      <c r="DF6" t="inlineStr"/>
+      <c r="DG6" t="inlineStr"/>
+      <c r="DH6" t="inlineStr"/>
+      <c r="DI6" t="inlineStr"/>
+      <c r="DJ6" t="inlineStr"/>
+      <c r="DK6" t="n">
+        <v>-0.1390740244736035</v>
+      </c>
+      <c r="DL6" t="n">
+        <v>0.2202469875888946</v>
+      </c>
+      <c r="DM6" t="n">
+        <v>-0.1412867372952507</v>
+      </c>
+      <c r="DN6" t="n">
+        <v>-0.03052835247181207</v>
+      </c>
+      <c r="DO6" t="n">
+        <v>-0.1186841637740814</v>
+      </c>
+      <c r="DP6" t="inlineStr"/>
+      <c r="DQ6" t="inlineStr"/>
+      <c r="DR6" t="inlineStr"/>
+      <c r="DS6" t="inlineStr"/>
+      <c r="DT6" t="inlineStr"/>
+      <c r="DU6" t="n">
+        <v>-0.1757684850489616</v>
+      </c>
+      <c r="DV6" t="n">
+        <v>-0.1759420071849851</v>
+      </c>
+      <c r="DW6" t="n">
+        <v>-0.1650090722933024</v>
+      </c>
+      <c r="DX6" t="n">
+        <v>-0.51615540723395</v>
+      </c>
+      <c r="DY6" t="n">
+        <v>-0.4382460251447453</v>
+      </c>
+      <c r="DZ6" t="n">
+        <v>-0.3978801748867733</v>
+      </c>
+      <c r="EA6" t="n">
+        <v>-0.2060018875339225</v>
+      </c>
+      <c r="EB6" t="n">
+        <v>-0.3110891182909645</v>
+      </c>
+      <c r="EC6" t="n">
+        <v>-0.1550738859356331</v>
+      </c>
+      <c r="ED6" t="n">
+        <v>-0.3373857089646695</v>
+      </c>
+      <c r="EE6" t="n">
+        <v>-0.3192233138118876</v>
+      </c>
+      <c r="EF6" t="inlineStr"/>
+      <c r="EG6" t="inlineStr"/>
+      <c r="EH6" t="inlineStr"/>
+      <c r="EI6" t="inlineStr"/>
+      <c r="EJ6" t="inlineStr"/>
+      <c r="EK6" t="inlineStr"/>
+      <c r="EL6" t="inlineStr"/>
+      <c r="EM6" t="inlineStr"/>
+      <c r="EN6" t="n">
+        <v>-0.6169415727856746</v>
+      </c>
+      <c r="EO6" t="inlineStr"/>
+      <c r="EP6" t="n">
+        <v>-0.2615200869695382</v>
+      </c>
+      <c r="EQ6" t="n">
+        <v>-0.2111889952281762</v>
+      </c>
+      <c r="ER6" t="inlineStr"/>
+      <c r="ES6" t="inlineStr"/>
+      <c r="ET6" t="n">
+        <v>-0.06969589500293782</v>
+      </c>
+      <c r="EU6" t="n">
+        <v>0.02160194095299506</v>
+      </c>
+      <c r="EV6" t="inlineStr"/>
+      <c r="EW6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>2023→2024</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>-0.2594317987974213</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-0.2729269936683725</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.2820727556756566</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.2592516517109376</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.2566714783295714</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-0.2646628224964847</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-0.2562875001663549</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.2717596929038475</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-0.2436278996769481</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-0.2643517051268098</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-0.2505252759115857</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-0.2796531252659626</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-0.2753921814493996</v>
+      </c>
+      <c r="O7" t="n">
+        <v>-0.2904834466992847</v>
+      </c>
+      <c r="P7" t="n">
+        <v>-0.3194412603704313</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>-0.2708066414075985</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-0.2925453598863923</v>
+      </c>
+      <c r="S7" t="n">
+        <v>-0.2654247077333203</v>
+      </c>
+      <c r="T7" t="n">
+        <v>-0.3019969931369371</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-0.2807388354686173</v>
+      </c>
+      <c r="V7" t="n">
+        <v>-0.2929871246814741</v>
+      </c>
+      <c r="W7" t="n">
+        <v>-0.3536365438496381</v>
+      </c>
+      <c r="X7" t="n">
+        <v>-0.3352366629062935</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>-0.325334975524374</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>-0.3241884612371706</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>-0.3352023214486941</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>-0.3356886352422705</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>-0.3370476642524149</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>-0.3768635871164179</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>-0.3784576909680712</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>-0.2910641223477528</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>-0.2803262196919674</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>-0.2805813111377402</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>-0.3134871600980702</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>-0.2791368261853435</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>-0.2273365840521624</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>-0.2864363668151855</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>-0.2933174597341983</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>-0.3355732226068184</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>-0.3414480257110393</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>-0.363230615771351</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>-0.3620364943668344</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>-0.3018968099778609</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>-0.3578183504873618</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>-0.3966744544118681</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>-0.1675787252807446</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>-0.130311507109969</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>-0.1375292916422852</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>-0.1676117072771399</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>-0.1821993032821752</v>
+      </c>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="n">
+        <v>-0.153346726078107</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>-0.1863475619121546</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>-0.2202087634041767</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>-0.268747218340474</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>-0.2392397881513437</v>
+      </c>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr"/>
+      <c r="BI7" t="inlineStr"/>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="n">
+        <v>-0.2150765872913096</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>-0.2250756615791447</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>-0.2062872995613052</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>-0.2232239466644783</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>-0.1623535545589156</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>-0.1866341379453189</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>-0.1843114197497089</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>-0.1468262956207678</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>-0.2181850941814183</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>-0.3493891003393941</v>
+      </c>
+      <c r="CB7" t="inlineStr"/>
+      <c r="CC7" t="n">
+        <v>0.08008899777067491</v>
+      </c>
+      <c r="CD7" t="inlineStr"/>
+      <c r="CE7" t="inlineStr"/>
+      <c r="CF7" t="n">
+        <v>-0.3094162540279157</v>
+      </c>
+      <c r="CG7" t="n">
+        <v>-0.2660813858513187</v>
+      </c>
+      <c r="CH7" t="n">
+        <v>-0.3530586626602386</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>-0.3274186434229494</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>-0.2166385755452307</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>-0.234663102775329</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>-0.2565165053098202</v>
+      </c>
+      <c r="CM7" t="n">
+        <v>-0.05030180475987756</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>-0.4409923066196937</v>
+      </c>
+      <c r="CO7" t="n">
+        <v>-0.1646780571551378</v>
+      </c>
+      <c r="CP7" t="n">
+        <v>-0.2265688268445052</v>
+      </c>
+      <c r="CQ7" t="n">
+        <v>-0.2876318891033227</v>
+      </c>
+      <c r="CR7" t="n">
+        <v>-0.09192994078378192</v>
+      </c>
+      <c r="CS7" t="inlineStr"/>
+      <c r="CT7" t="inlineStr"/>
+      <c r="CU7" t="inlineStr"/>
+      <c r="CV7" t="n">
+        <v>-0.1295895745169613</v>
+      </c>
+      <c r="CW7" t="n">
+        <v>0.2551738348402912</v>
+      </c>
+      <c r="CX7" t="n">
+        <v>0.1502750945962621</v>
+      </c>
+      <c r="CY7" t="inlineStr"/>
+      <c r="CZ7" t="n">
+        <v>-0.2814261451203137</v>
+      </c>
+      <c r="DA7" t="inlineStr"/>
+      <c r="DB7" t="inlineStr"/>
+      <c r="DC7" t="inlineStr"/>
+      <c r="DD7" t="inlineStr"/>
+      <c r="DE7" t="inlineStr"/>
+      <c r="DF7" t="inlineStr"/>
+      <c r="DG7" t="inlineStr"/>
+      <c r="DH7" t="inlineStr"/>
+      <c r="DI7" t="inlineStr"/>
+      <c r="DJ7" t="n">
+        <v>0.2829814253805294</v>
+      </c>
+      <c r="DK7" t="n">
+        <v>-0.04358865132269951</v>
+      </c>
+      <c r="DL7" t="n">
+        <v>0.01027897002867739</v>
+      </c>
+      <c r="DM7" t="n">
+        <v>-0.08824051349127782</v>
+      </c>
+      <c r="DN7" t="n">
+        <v>0.08163264411826088</v>
+      </c>
+      <c r="DO7" t="n">
+        <v>-0.2395005099237011</v>
+      </c>
+      <c r="DP7" t="n">
+        <v>-0.1332583837500385</v>
+      </c>
+      <c r="DQ7" t="n">
+        <v>-0.01634389849952633</v>
+      </c>
+      <c r="DR7" t="n">
+        <v>0.4517561785635378</v>
+      </c>
+      <c r="DS7" t="n">
+        <v>-0.2446430962845483</v>
+      </c>
+      <c r="DT7" t="n">
+        <v>-0.02325571490767775</v>
+      </c>
+      <c r="DU7" t="n">
+        <v>-0.05285541960081819</v>
+      </c>
+      <c r="DV7" t="n">
+        <v>-0.06105111185564471</v>
+      </c>
+      <c r="DW7" t="n">
+        <v>0.1021158152244483</v>
+      </c>
+      <c r="DX7" t="n">
+        <v>-0.121074901640684</v>
+      </c>
+      <c r="DY7" t="n">
+        <v>-0.1416272084110419</v>
+      </c>
+      <c r="DZ7" t="n">
+        <v>-0.33946334599315</v>
+      </c>
+      <c r="EA7" t="n">
+        <v>-0.3473814932989416</v>
+      </c>
+      <c r="EB7" t="n">
+        <v>-0.4180005185020645</v>
+      </c>
+      <c r="EC7" t="n">
+        <v>-0.4013696393398343</v>
+      </c>
+      <c r="ED7" t="n">
+        <v>-0.3467475068249986</v>
+      </c>
+      <c r="EE7" t="n">
+        <v>-0.3627689902253817</v>
+      </c>
+      <c r="EF7" t="n">
+        <v>-0.3259340687631367</v>
+      </c>
+      <c r="EG7" t="n">
+        <v>-0.2950583335972645</v>
+      </c>
+      <c r="EH7" t="n">
+        <v>-0.2410519625274192</v>
+      </c>
+      <c r="EI7" t="n">
+        <v>-0.2709573336247377</v>
+      </c>
+      <c r="EJ7" t="inlineStr"/>
+      <c r="EK7" t="inlineStr"/>
+      <c r="EL7" t="inlineStr"/>
+      <c r="EM7" t="inlineStr"/>
+      <c r="EN7" t="n">
+        <v>-0.07962153920591675</v>
+      </c>
+      <c r="EO7" t="n">
+        <v>-0.3489122880116122</v>
+      </c>
+      <c r="EP7" t="n">
+        <v>-0.4674649223308158</v>
+      </c>
+      <c r="EQ7" t="n">
+        <v>-0.5285323906780812</v>
+      </c>
+      <c r="ER7" t="n">
+        <v>-0.04320340802328637</v>
+      </c>
+      <c r="ES7" t="n">
+        <v>-0.2162193039551035</v>
+      </c>
+      <c r="ET7" t="n">
+        <v>-0.4526044357330425</v>
+      </c>
+      <c r="EU7" t="n">
+        <v>-0.5651343328895253</v>
+      </c>
+      <c r="EV7" t="inlineStr"/>
+      <c r="EW7" t="n">
+        <v>-0.2318632866559778</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>2024→2025</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>-0.1551803852564326</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-0.1351282821875728</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-0.1312168433216456</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-0.1478038409274456</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.1540998474470214</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.1345858202688994</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-0.1451405885827874</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.136646139677091</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-0.1398018006391775</v>
+      </c>
+      <c r="K8" t="n">
+        <v>-0.194062925698228</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-0.2258956734849669</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-0.2286261336494855</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-0.1877019518625787</v>
+      </c>
+      <c r="O8" t="n">
+        <v>-0.1857452464790574</v>
+      </c>
+      <c r="P8" t="n">
+        <v>-0.2197723802361802</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>-0.14987818954347</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-0.1284283644889577</v>
+      </c>
+      <c r="S8" t="n">
+        <v>-0.127522989681923</v>
+      </c>
+      <c r="T8" t="n">
+        <v>-0.2094900306164202</v>
+      </c>
+      <c r="U8" t="n">
+        <v>-0.2351702702780818</v>
+      </c>
+      <c r="V8" t="n">
+        <v>-0.1908414541622632</v>
+      </c>
+      <c r="W8" t="n">
+        <v>-0.2695064723679099</v>
+      </c>
+      <c r="X8" t="n">
+        <v>-0.2810875030931665</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>-0.2879607660037964</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>-0.2170198433516113</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>-0.2380693985669513</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>-0.289395749106208</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>-0.2073776179390503</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>-0.2400898113123775</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>-0.2562446003753207</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>-0.2441893731377363</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>-0.2283027670225799</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>-0.1810161426688701</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>-0.2854351186712245</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>-0.2753565794150292</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>-0.253551781196073</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>-0.2534302108412305</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>-0.2384634661115665</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>-0.15581927954773</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>-0.2711975119934431</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>-0.2756089931141643</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>-0.3008051632538367</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>-0.2565708570461185</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>-0.1955733191939473</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>-0.205262588362535</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>-0.2292579482833146</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>-0.2183648494063064</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>-0.2700554731091156</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>-0.2052668304219125</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>-0.2060816983768436</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>-0.1734778561720578</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>-0.2097867750309286</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>-0.223086999824063</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>-0.2323786374476908</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>-0.2750609459522826</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>-0.3379445493527173</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>-0.1021448663437239</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>-0.1140262754156538</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>-0.1492622620306898</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>-0.1562909957186038</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>-0.154687236723051</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>-0.1740821905970416</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>-0.1858095895938083</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>-0.2239505681567007</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>-0.08637630409691344</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>-0.1619813662509451</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>-0.04549072976756019</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>0.001426784497789768</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>-0.1244477536832544</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>-0.08495825555521641</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>-0.08388148398070161</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>-0.08842211534549893</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>-0.1258304319486303</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>-0.09478470106154369</v>
+      </c>
+      <c r="BX8" t="n">
+        <v>-0.05052421751025626</v>
+      </c>
+      <c r="BY8" t="n">
+        <v>-0.1293794423533772</v>
+      </c>
+      <c r="BZ8" t="n">
+        <v>-0.06133901267663688</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>-0.08511756682120186</v>
+      </c>
+      <c r="CB8" t="n">
+        <v>-0.3397179731526814</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>-0.01419934233881204</v>
+      </c>
+      <c r="CD8" t="inlineStr"/>
+      <c r="CE8" t="n">
+        <v>-0.1009341451519781</v>
+      </c>
+      <c r="CF8" t="n">
+        <v>-0.1288386769032401</v>
+      </c>
+      <c r="CG8" t="n">
+        <v>0.01567061648377699</v>
+      </c>
+      <c r="CH8" t="n">
+        <v>0.1099585459110202</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>-0.1274453211192439</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>-0.1086945989245827</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>0.03552588996845341</v>
+      </c>
+      <c r="CL8" t="n">
+        <v>-0.5231564017929484</v>
+      </c>
+      <c r="CM8" t="inlineStr"/>
+      <c r="CN8" t="n">
+        <v>0.05490583740122723</v>
+      </c>
+      <c r="CO8" t="n">
+        <v>-0.09248502820703131</v>
+      </c>
+      <c r="CP8" t="n">
+        <v>-0.0255858413361203</v>
+      </c>
+      <c r="CQ8" t="n">
+        <v>-0.003245590429647116</v>
+      </c>
+      <c r="CR8" t="n">
+        <v>-0.4329870773374971</v>
+      </c>
+      <c r="CS8" t="inlineStr"/>
+      <c r="CT8" t="inlineStr"/>
+      <c r="CU8" t="inlineStr"/>
+      <c r="CV8" t="n">
+        <v>0.03612250773056935</v>
+      </c>
+      <c r="CW8" t="n">
+        <v>0.1488947079357645</v>
+      </c>
+      <c r="CX8" t="n">
+        <v>0.03706876818899119</v>
+      </c>
+      <c r="CY8" t="inlineStr"/>
+      <c r="CZ8" t="n">
+        <v>0.01702084481384958</v>
+      </c>
+      <c r="DA8" t="n">
+        <v>0.03739788241290753</v>
+      </c>
+      <c r="DB8" t="n">
+        <v>-0.05388891022055731</v>
+      </c>
+      <c r="DC8" t="n">
+        <v>-0.1026134472653935</v>
+      </c>
+      <c r="DD8" t="inlineStr"/>
+      <c r="DE8" t="n">
+        <v>-0.2487735890008311</v>
+      </c>
+      <c r="DF8" t="inlineStr"/>
+      <c r="DG8" t="inlineStr"/>
+      <c r="DH8" t="inlineStr"/>
+      <c r="DI8" t="inlineStr"/>
+      <c r="DJ8" t="n">
+        <v>0.01330559696204592</v>
+      </c>
+      <c r="DK8" t="inlineStr"/>
+      <c r="DL8" t="n">
+        <v>0.01284496162253568</v>
+      </c>
+      <c r="DM8" t="n">
+        <v>-0.05964868017717073</v>
+      </c>
+      <c r="DN8" t="n">
+        <v>0.1744689530641921</v>
+      </c>
+      <c r="DO8" t="n">
+        <v>0.0491471401383361</v>
+      </c>
+      <c r="DP8" t="inlineStr"/>
+      <c r="DQ8" t="inlineStr"/>
+      <c r="DR8" t="n">
+        <v>-0.2739076233468278</v>
+      </c>
+      <c r="DS8" t="n">
+        <v>-0.2551418603072637</v>
+      </c>
+      <c r="DT8" t="n">
+        <v>0.1826345522308586</v>
+      </c>
+      <c r="DU8" t="n">
+        <v>-0.09692897716813587</v>
+      </c>
+      <c r="DV8" t="n">
+        <v>-0.07962060889158451</v>
+      </c>
+      <c r="DW8" t="n">
+        <v>0.1614340235381837</v>
+      </c>
+      <c r="DX8" t="n">
+        <v>-0.06677203002051346</v>
+      </c>
+      <c r="DY8" t="n">
+        <v>-0.08568545509330239</v>
+      </c>
+      <c r="DZ8" t="n">
+        <v>-0.1618944333852399</v>
+      </c>
+      <c r="EA8" t="n">
+        <v>-0.1461247276191413</v>
+      </c>
+      <c r="EB8" t="n">
+        <v>-0.142601100850821</v>
+      </c>
+      <c r="EC8" t="n">
+        <v>-0.1158132938466423</v>
+      </c>
+      <c r="ED8" t="n">
+        <v>-0.1684085976357554</v>
+      </c>
+      <c r="EE8" t="n">
+        <v>-0.1595587254233637</v>
+      </c>
+      <c r="EF8" t="n">
+        <v>-0.1712658433441705</v>
+      </c>
+      <c r="EG8" t="n">
+        <v>-0.1604996725789256</v>
+      </c>
+      <c r="EH8" t="n">
+        <v>-0.1676828325418098</v>
+      </c>
+      <c r="EI8" t="n">
+        <v>-0.2488601847705558</v>
+      </c>
+      <c r="EJ8" t="n">
+        <v>0.03709796694584355</v>
+      </c>
+      <c r="EK8" t="n">
+        <v>-0.03313055054897074</v>
+      </c>
+      <c r="EL8" t="n">
+        <v>-0.1405540085693708</v>
+      </c>
+      <c r="EM8" t="n">
+        <v>-0.07995738166363608</v>
+      </c>
+      <c r="EN8" t="n">
+        <v>0.05226066486768133</v>
+      </c>
+      <c r="EO8" t="n">
+        <v>-0.2534073388905993</v>
+      </c>
+      <c r="EP8" t="n">
+        <v>-0.01577692190979718</v>
+      </c>
+      <c r="EQ8" t="n">
+        <v>-0.1528868297985992</v>
+      </c>
+      <c r="ER8" t="n">
+        <v>-0.1094870672180255</v>
+      </c>
+      <c r="ES8" t="n">
+        <v>-0.09853999531804636</v>
+      </c>
+      <c r="ET8" t="n">
+        <v>-0.1638616557078931</v>
+      </c>
+      <c r="EU8" t="n">
+        <v>0.02313712924011391</v>
+      </c>
+      <c r="EV8" t="n">
+        <v>-0.09756723586969951</v>
+      </c>
+      <c r="EW8" t="n">
+        <v>-0.179062688905379</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>